<commit_message>
English-language release for PeerJ Computer Science
- File, sheet, column, and categorical-value names translated from Korean; DATA_CODEBOOK.md maps every English name to its Korean original
- README rewritten (usage, requirements, citation); requirements.txt and .gitignore added
- No change to numerical values or analysis logic: the CPU-only reproduction (README step 3) re-run on this version regenerated every result table with zero numeric differences and byte-identical R11 figures

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/audit/R11_adjudication_sheets.xlsx
+++ b/audit/R11_adjudication_sheets.xlsx
@@ -7,9 +7,9 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="읽어주세요" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="① 독립 재평가 120" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="② 합의 판정 40" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read me" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="① Independent reannotation 120" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="② Consensus adjudication 40" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -195,7 +195,7 @@
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hang" typeface="Malgun Gothic"/>
         <a:font script="Hans" typeface="宋体"/>
         <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Times New Roman"/>
@@ -229,7 +229,7 @@
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hang" typeface="Malgun Gothic"/>
         <a:font script="Hans" typeface="宋体"/>
         <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Arial"/>
@@ -446,35 +446,35 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>R11 판정 키트 — 먼저 00_판정기준_codebook.md 를 읽으세요.</t>
+          <t>R11 adjudication kit: read the codebook (R11_codebook.md, adjudication criteria) first.</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>시트 ① (독립 재평가): 120건 전부. 원래 판정은 보이지 않습니다. 다른 사람과 상의하지 마세요. 노란 칸에 1/2/3 과 규칙 번호(R1~R10).</t>
+          <t>Sheet ① (independent re-annotation): all 120 items. The original judgments are hidden. Do not discuss with anyone. Enter 1/2/3 and the rule number (R1-R10) in the yellow cells.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>시트 ② (합의 판정): 원래 3인 판정이 갈린 40건. 원래 판정을 보고, 코드북 규칙을 근거로 최종 범주를 정합니다.</t>
+          <t>Sheet ② (consensus adjudication): the 40 items on which the original three annotators disagreed. Look at the original judgments and decide the final class based on the codebook rules.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>시트 ①은 평가자마다 파일을 복사해 따로 작성(파일명 끝에 _평가자1, _평가자2). 시트 ②는 판정자 1인 또는 2인 합의로 한 파일.</t>
+          <t>Sheet ①: each rater fills in a separate copy of the file (file name ending in _rater1, _rater2). Sheet ②: one file, by a single adjudicator or by consensus of two.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>판정 근거는 저장소 이름·설명·태그가 1순위, 부족하면 링크의 README 첫 화면까지만.</t>
+          <t>Basis for judgment: repository name, description and tags first; if insufficient, look only at the first screen of the README via the link.</t>
         </is>
       </c>
     </row>
@@ -506,7 +506,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>번호</t>
+          <t>item_no</t>
         </is>
       </c>
       <c r="B1" s="2" t="inlineStr">
@@ -516,17 +516,17 @@
       </c>
       <c r="C1" s="2" t="inlineStr">
         <is>
-          <t>링크</t>
+          <t>Link</t>
         </is>
       </c>
       <c r="D1" s="2" t="inlineStr">
         <is>
-          <t>한글 설명</t>
+          <t>Short description</t>
         </is>
       </c>
       <c r="E1" s="2" t="inlineStr">
         <is>
-          <t>description (원문)</t>
+          <t>description (original)</t>
         </is>
       </c>
       <c r="F1" s="2" t="inlineStr">
@@ -536,17 +536,17 @@
       </c>
       <c r="G1" s="2" t="inlineStr">
         <is>
-          <t>판정(1/2/3)</t>
+          <t>Judgment (1/2/3)</t>
         </is>
       </c>
       <c r="H1" s="2" t="inlineStr">
         <is>
-          <t>규칙 번호</t>
+          <t>Rule no.</t>
         </is>
       </c>
       <c r="I1" s="2" t="inlineStr">
         <is>
-          <t>메모</t>
+          <t>Notes</t>
         </is>
       </c>
     </row>
@@ -566,7 +566,7 @@
       </c>
       <c r="D2" s="1" t="inlineStr">
         <is>
-          <t>기업 소프트웨어 자동화를 위한 AI 에이전트</t>
+          <t>An AI agent for automating enterprise software</t>
         </is>
       </c>
       <c r="E2" s="1" t="inlineStr">
@@ -597,7 +597,7 @@
       </c>
       <c r="D3" s="1" t="inlineStr">
         <is>
-          <t>데이터 분석 전 과정을 간소화하는 LLM 기반 AI 에이전트</t>
+          <t>An LLM-based AI agent that streamlines the entire data-analysis process</t>
         </is>
       </c>
       <c r="E3" s="1" t="inlineStr">
@@ -630,7 +630,7 @@
       </c>
       <c r="D4" s="1" t="inlineStr">
         <is>
-          <t>여러 AI 코딩 에이전트(Claude·Gemini·Codex·Cursor)를 명세 기반으로 오케스트레이션하는 CLI</t>
+          <t>A CLI that orchestrates multiple AI coding agents (Claude, Gemini, Codex, Cursor) from specifications</t>
         </is>
       </c>
       <c r="E4" s="1" t="inlineStr">
@@ -663,7 +663,7 @@
       </c>
       <c r="D5" s="1" t="inlineStr">
         <is>
-          <t>Claude 에이전트 스킬을 만드는 CLI(점진적 공개 검증). Claude Code가 스킬 생성 요청 시 사용</t>
+          <t>A CLI for creating Claude agent skills (with progressive-disclosure validation). Used by Claude Code when asked to create a skill</t>
         </is>
       </c>
       <c r="E5" s="1" t="inlineStr">
@@ -696,7 +696,7 @@
       </c>
       <c r="D6" s="1" t="inlineStr">
         <is>
-          <t>실무용 n8n 자동화 워크플로 9종 모음 — WhatsApp 에이전트, RAG 챗봇, 감성분석, 이메일 자동화, Airtable, 벡터 DB 파이프라인</t>
+          <t>A collection of 9 production n8n automation workflows - WhatsApp agent, RAG chatbot, sentiment analysis, email automation, Airtable, vector DB pipeline</t>
         </is>
       </c>
       <c r="E6" s="1" t="inlineStr">
@@ -729,7 +729,7 @@
       </c>
       <c r="D7" s="1" t="inlineStr">
         <is>
-          <t>Thordata 공식 개발자 포털 — 프록시 인프라·웹 데이터 도구·SDK·튜토리얼·AI 연동 개요</t>
+          <t>Thordata official developer portal - overview of proxy infrastructure, web data tools, SDKs, tutorials, and AI integrations</t>
         </is>
       </c>
       <c r="E7" s="1" t="inlineStr">
@@ -762,7 +762,7 @@
       </c>
       <c r="D8" s="1" t="inlineStr">
         <is>
-          <t>대규모로 웹을 검색·스크랩·상호작용하는 컨텍스트 API</t>
+          <t>A context API for searching, scraping, and interacting with the web at scale</t>
         </is>
       </c>
       <c r="E8" s="1" t="inlineStr">
@@ -795,7 +795,7 @@
       </c>
       <c r="D9" s="1" t="inlineStr">
         <is>
-          <t>탐색적 브라우저 테스트용 AI 에이전트</t>
+          <t>An AI agent for exploratory browser testing</t>
         </is>
       </c>
       <c r="E9" s="1" t="inlineStr">
@@ -828,7 +828,7 @@
       </c>
       <c r="D10" s="1" t="inlineStr">
         <is>
-          <t>PHP 프로젝트용 에이전트 스킬 배포·관리 Composer 플러그인</t>
+          <t>A Composer plugin for distributing and managing agent skills for PHP projects</t>
         </is>
       </c>
       <c r="E10" s="1" t="inlineStr">
@@ -861,7 +861,7 @@
       </c>
       <c r="D11" s="1" t="inlineStr">
         <is>
-          <t>에디터 안의 AI 개발팀 — 전문 에이전트 약 48개와 승인 게이트가 있는 워크플로. Claude Code·Cursor·Kiro·VS Code 지원</t>
+          <t>An AI development team inside the editor - about 48 specialized agents and workflows with approval gates. Supports Claude Code, Cursor, Kiro, VS Code</t>
         </is>
       </c>
       <c r="E11" s="1" t="inlineStr">
@@ -894,7 +894,7 @@
       </c>
       <c r="D12" s="1" t="inlineStr">
         <is>
-          <t>agentic-obs — OBS WebSocket API로 AI 어시스턴트가 OBS Studio(장면·소스·녹화·스트리밍)를 제어하게 하는 MCP 서버</t>
+          <t>agentic-obs - an MCP server that lets AI assistants control OBS Studio (scenes, sources, recording, streaming) through the OBS WebSocket API</t>
         </is>
       </c>
       <c r="E12" s="1" t="inlineStr">
@@ -927,7 +927,7 @@
       </c>
       <c r="D13" s="1" t="inlineStr">
         <is>
-          <t>Claude Code용 자율 리서치 에이전트 — 배경에서 조사해 유용한 맥락을 주입</t>
+          <t>An autonomous research agent for Claude Code - researches in the background and injects useful context</t>
         </is>
       </c>
       <c r="E13" s="1" t="inlineStr">
@@ -960,7 +960,7 @@
       </c>
       <c r="D14" s="1" t="inlineStr">
         <is>
-          <t>맞춤 에이전트 기능과 서브에이전트로 Claude Code를 만능 AI 에이전트로 만들기</t>
+          <t>Turning Claude Code into an all-purpose AI agent with custom agent features and sub-agents</t>
         </is>
       </c>
       <c r="E14" s="1" t="inlineStr">
@@ -991,7 +991,7 @@
       </c>
       <c r="D15" s="1" t="inlineStr">
         <is>
-          <t>데스크톱용 보이지 않는 AI 에이전트</t>
+          <t>An invisible AI agent for the desktop</t>
         </is>
       </c>
       <c r="E15" s="1" t="inlineStr">
@@ -1022,7 +1022,7 @@
       </c>
       <c r="D16" s="1" t="inlineStr">
         <is>
-          <t>ToRA — 도구와 상호작용해 어려운 수학 추론 문제를 푸는 도구통합 LLM 에이전트 시리즈(ICLR'24 논문)</t>
+          <t>ToRA - a series of tool-integrated LLM agents that solve hard mathematical reasoning problems by interacting with tools (ICLR'24 paper)</t>
         </is>
       </c>
       <c r="E16" s="1" t="inlineStr">
@@ -1055,7 +1055,7 @@
       </c>
       <c r="D17" s="1" t="inlineStr">
         <is>
-          <t>devcontainer.json 설정으로 개발 컨테이너를 생성·구성하는 MCP 서버</t>
+          <t>An MCP server that creates and configures development containers from devcontainer.json settings</t>
         </is>
       </c>
       <c r="E17" s="1" t="inlineStr">
@@ -1088,7 +1088,7 @@
       </c>
       <c r="D18" s="1" t="inlineStr">
         <is>
-          <t>Ghidra와 LLM 에이전트를 조율해 바이너리 분석(리버스 엔지니어링)을 자동화</t>
+          <t>Automating binary analysis (reverse engineering) by coordinating Ghidra and LLM agents</t>
         </is>
       </c>
       <c r="E18" s="1" t="inlineStr">
@@ -1121,7 +1121,7 @@
       </c>
       <c r="D19" s="1" t="inlineStr">
         <is>
-          <t>'엿듣는 LLM 에이전트' 기반 오픈소스 AI 의료 음성 어시스턴트</t>
+          <t>An open-source AI medical voice assistant based on an 'eavesdropping LLM agent'</t>
         </is>
       </c>
       <c r="E19" s="1" t="inlineStr">
@@ -1152,7 +1152,7 @@
       </c>
       <c r="D20" s="1" t="inlineStr">
         <is>
-          <t>AI 에이전트 워크숍용 실습(랩) 저장소</t>
+          <t>A hands-on lab repository for an AI agent workshop</t>
         </is>
       </c>
       <c r="E20" s="1" t="inlineStr">
@@ -1183,7 +1183,7 @@
       </c>
       <c r="D21" s="1" t="inlineStr">
         <is>
-          <t>autogen을 이용한 실험 모음</t>
+          <t>A collection of experiments using autogen</t>
         </is>
       </c>
       <c r="E21" s="1" t="inlineStr">
@@ -1214,7 +1214,7 @@
       </c>
       <c r="D22" s="1" t="inlineStr">
         <is>
-          <t>DevOps 중심 MCP 서버 정리 목록 — 소스관리·IaC·쿠버네티스·CI/CD·클라우드·관측·보안 등</t>
+          <t>A curated list of DevOps-focused MCP servers - source control, IaC, Kubernetes, CI/CD, cloud, observability, security, etc.</t>
         </is>
       </c>
       <c r="E22" s="1" t="inlineStr">
@@ -1247,7 +1247,7 @@
       </c>
       <c r="D23" s="1" t="inlineStr">
         <is>
-          <t>TheraBot — SaaS형 AI 정신건강 동반자. 공감형 챗봇, 치료사 예약, 에이전트가 만드는 환자 요약</t>
+          <t>TheraBot - an AI mental-health companion as SaaS. Empathetic chatbot, therapist booking, patient summaries generated by agents</t>
         </is>
       </c>
       <c r="E23" s="1" t="inlineStr">
@@ -1280,7 +1280,7 @@
       </c>
       <c r="D24" s="1" t="inlineStr">
         <is>
-          <t>Claude Code CLI로 코딩할 때 쓰는 도구 모음. 코드베이스 의미 색인 기반 검색(smartgrep)과 코드베이스 큐레이터 Claude 포함</t>
+          <t>A tool collection for coding with the Claude Code CLI. Includes semantic-index-based codebase search (smartgrep) and a codebase-curator Claude</t>
         </is>
       </c>
       <c r="E24" s="1" t="inlineStr">
@@ -1313,7 +1313,7 @@
       </c>
       <c r="D25" s="1" t="inlineStr">
         <is>
-          <t>Simli WebRTC AI 에이전트 데모</t>
+          <t>Simli WebRTC AI agent demo</t>
         </is>
       </c>
       <c r="E25" s="1" t="inlineStr">
@@ -1344,7 +1344,7 @@
       </c>
       <c r="D26" s="1" t="inlineStr">
         <is>
-          <t>Letta SDK(TypeScript·Python) 코드 스니펫 — 상태 유지 AI 에이전트 개발용</t>
+          <t>Code snippets for the Letta SDK (TypeScript, Python) - for developing stateful AI agents</t>
         </is>
       </c>
       <c r="E26" s="1" t="inlineStr">
@@ -1377,7 +1377,7 @@
       </c>
       <c r="D27" s="1" t="inlineStr">
         <is>
-          <t>MCP 서버 개발용 TypeScript 스타터 템플릿</t>
+          <t>A TypeScript starter template for developing MCP servers</t>
         </is>
       </c>
       <c r="E27" s="1" t="inlineStr">
@@ -1410,7 +1410,7 @@
       </c>
       <c r="D28" s="1" t="inlineStr">
         <is>
-          <t>Magento 2 개발용으로 설계된 Claude Code 서브에이전트 모음</t>
+          <t>A collection of Claude Code sub-agents designed for Magento 2 development</t>
         </is>
       </c>
       <c r="E28" s="1" t="inlineStr">
@@ -1443,7 +1443,7 @@
       </c>
       <c r="D29" s="1" t="inlineStr">
         <is>
-          <t>LLM 파이프라인과 AI 에이전트</t>
+          <t>LLM pipelines and AI agents</t>
         </is>
       </c>
       <c r="E29" s="1" t="inlineStr">
@@ -1474,7 +1474,7 @@
       </c>
       <c r="D30" s="1" t="inlineStr">
         <is>
-          <t>실행 가능한 AI 프롬프트·로직·데이터를 담는 모듈형 파일 형식</t>
+          <t>A modular file format that holds executable AI prompts, logic, and data</t>
         </is>
       </c>
       <c r="E30" s="1" t="inlineStr">
@@ -1507,7 +1507,7 @@
       </c>
       <c r="D31" s="1" t="inlineStr">
         <is>
-          <t>🐧 작업 중… (내용 없음)</t>
+          <t>🐧 Work in progress… (no content)</t>
         </is>
       </c>
       <c r="E31" s="1" t="inlineStr">
@@ -1540,7 +1540,7 @@
       </c>
       <c r="D32" s="1" t="inlineStr">
         <is>
-          <t>AI 에이전트용 멀티 런타임 자동화 인프라 — 네이티브 CDP 브라우저 제어, 레시피 시스템, 실행 컨텍스트 관리</t>
+          <t>Multi-runtime automation infrastructure for AI agents - native CDP browser control, recipe system, execution-context management</t>
         </is>
       </c>
       <c r="E32" s="1" t="inlineStr">
@@ -1573,7 +1573,7 @@
       </c>
       <c r="D33" s="1" t="inlineStr">
         <is>
-          <t>Omnimesh — 에이전트와 서비스의 범용 네트워크</t>
+          <t>Omnimesh - a universal network of agents and services</t>
         </is>
       </c>
       <c r="E33" s="1" t="inlineStr">
@@ -1606,7 +1606,7 @@
       </c>
       <c r="D34" s="1" t="inlineStr">
         <is>
-          <t>AI 에이전트·MCP·AI 워크플로 자동화 모음(AI 에이전트용 MCP 서버 약 400개)</t>
+          <t>A collection of AI agents, MCP, and AI workflow automation (about 400 MCP servers for AI agents)</t>
         </is>
       </c>
       <c r="E34" s="1" t="inlineStr">
@@ -1639,7 +1639,7 @@
       </c>
       <c r="D35" s="1" t="inlineStr">
         <is>
-          <t>OpenMemory — 독자적 인지 아키텍처로 장기 기억 저장·회상·설명을 AI에 추가</t>
+          <t>OpenMemory - adds long-term memory storage, recall, and explanation to AI with its own cognitive architecture</t>
         </is>
       </c>
       <c r="E35" s="1" t="inlineStr">
@@ -1672,7 +1672,7 @@
       </c>
       <c r="D36" s="1" t="inlineStr">
         <is>
-          <t>TianGong-Agent (설명 없음)</t>
+          <t>TianGong-Agent (no description)</t>
         </is>
       </c>
       <c r="E36" s="1" t="inlineStr">
@@ -1703,7 +1703,7 @@
       </c>
       <c r="D37" s="1" t="inlineStr">
         <is>
-          <t>Anthropic 스킬을 Cursor IDE에 통합하는 프레임워크 — 에이전트가 전문 지식을 일관되게 적용</t>
+          <t>A framework that integrates Anthropic skills into the Cursor IDE - agents apply specialized knowledge consistently</t>
         </is>
       </c>
       <c r="E37" s="1" t="inlineStr">
@@ -1734,7 +1734,7 @@
       </c>
       <c r="D38" s="1" t="inlineStr">
         <is>
-          <t>AI 에이전트용으로 만든 훅(hook) 모음</t>
+          <t>A collection of hooks made for AI agents</t>
         </is>
       </c>
       <c r="E38" s="1" t="inlineStr">
@@ -1765,7 +1765,7 @@
       </c>
       <c r="D39" s="1" t="inlineStr">
         <is>
-          <t>논문 코드: 팝업으로 비전-언어 컴퓨터 에이전트를 공격하기</t>
+          <t>Paper code: attacking vision-language computer agents with pop-ups</t>
         </is>
       </c>
       <c r="E39" s="1" t="inlineStr">
@@ -1798,7 +1798,7 @@
       </c>
       <c r="D40" s="1" t="inlineStr">
         <is>
-          <t>elizaos/eliza, swarms AI 에이전트를 배포하는 Terraform 프레임워크</t>
+          <t>A Terraform framework for deploying elizaos/eliza and swarms AI agents</t>
         </is>
       </c>
       <c r="E40" s="1" t="inlineStr">
@@ -1831,7 +1831,7 @@
       </c>
       <c r="D41" s="1" t="inlineStr">
         <is>
-          <t>온체인 에이전트 마켓플레이스 — 누구나 AI 에이전트를 발견·배포·수익화</t>
+          <t>An on-chain agent marketplace - anyone can discover, deploy, and monetize AI agents</t>
         </is>
       </c>
       <c r="E41" s="1" t="inlineStr">
@@ -1862,7 +1862,7 @@
       </c>
       <c r="D42" s="1" t="inlineStr">
         <is>
-          <t>커넥터 30개 이상 내장, AI 에이전트를 만드는 .NET 라이브러리</t>
+          <t>A .NET library for building AI agents, with more than 30 built-in connectors</t>
         </is>
       </c>
       <c r="E42" s="1" t="inlineStr">
@@ -1895,7 +1895,7 @@
       </c>
       <c r="D43" s="1" t="inlineStr">
         <is>
-          <t>PydanticAI와 Permit.io 세밀 권한 프레임워크로 안전한 AI 에이전트를 구현하는 시연(데모)</t>
+          <t>A demonstration (demo) of building secure AI agents with PydanticAI and the Permit.io fine-grained authorization framework</t>
         </is>
       </c>
       <c r="E43" s="1" t="inlineStr">
@@ -1928,7 +1928,7 @@
       </c>
       <c r="D44" s="1" t="inlineStr">
         <is>
-          <t>AST 기반 AI 개발 에이전트 — Django/Flask 자율 빌더, 제로 토큰, 샌드박스(인도 제작)</t>
+          <t>An AST-based AI development agent - autonomous Django/Flask builder, zero tokens, sandbox (made in India)</t>
         </is>
       </c>
       <c r="E44" s="1" t="inlineStr">
@@ -1961,7 +1961,7 @@
       </c>
       <c r="D45" s="1" t="inlineStr">
         <is>
-          <t>기업급 멀티에이전트 오케스트레이션 프레임워크(swarms.ai)</t>
+          <t>Enterprise-grade multi-agent orchestration framework (swarms.ai)</t>
         </is>
       </c>
       <c r="E45" s="1" t="inlineStr">
@@ -1994,7 +1994,7 @@
       </c>
       <c r="D46" s="1" t="inlineStr">
         <is>
-          <t>ICLR 2026 논문: Agent-X — 시각 중심 에이전트 과제의 멀티모달 추론 평가</t>
+          <t>ICLR 2026 paper: Agent-X - evaluating multimodal reasoning on vision-centric agent tasks</t>
         </is>
       </c>
       <c r="E46" s="1" t="inlineStr">
@@ -2027,7 +2027,7 @@
       </c>
       <c r="D47" s="1" t="inlineStr">
         <is>
-          <t>Waffy — 웹용 AI 코파일럿</t>
+          <t>Waffy - an AI copilot for the web</t>
         </is>
       </c>
       <c r="E47" s="1" t="inlineStr">
@@ -2060,7 +2060,7 @@
       </c>
       <c r="D48" s="1" t="inlineStr">
         <is>
-          <t>Go 언어 AI 에이전트 프레임워크</t>
+          <t>An AI agent framework in the Go language</t>
         </is>
       </c>
       <c r="E48" s="1" t="inlineStr">
@@ -2091,7 +2091,7 @@
       </c>
       <c r="D49" s="1" t="inlineStr">
         <is>
-          <t>F# interactive(fsi)를 감싸 AI 에이전트용 MCP 서버 엔드포인트를 노출하는 래퍼</t>
+          <t>A wrapper around F# interactive (fsi) that exposes an MCP server endpoint for AI agents</t>
         </is>
       </c>
       <c r="E49" s="1" t="inlineStr">
@@ -2122,7 +2122,7 @@
       </c>
       <c r="D50" s="1" t="inlineStr">
         <is>
-          <t>LangGraph와 멀티에이전트 컨트롤 플레인으로 목표 지향 멀티에이전트 시스템을 만드는 에이전트 AI 프레임워크</t>
+          <t>An agentic AI framework for building goal-oriented multi-agent systems with LangGraph and a multi-agent control plane</t>
         </is>
       </c>
       <c r="E50" s="1" t="inlineStr">
@@ -2155,7 +2155,7 @@
       </c>
       <c r="D51" s="1" t="inlineStr">
         <is>
-          <t>AI 에이전트가 클래시 로얄을 자율 플레이. Claude Code+멀티에이전트로 트위치 생방송에서 1000 트로피 달성</t>
+          <t>An AI agent plays Clash Royale autonomously. Reached 1,000 trophies on a Twitch live stream with Claude Code + multiple agents</t>
         </is>
       </c>
       <c r="E51" s="1" t="inlineStr">
@@ -2188,7 +2188,7 @@
       </c>
       <c r="D52" s="1" t="inlineStr">
         <is>
-          <t>AI 에이전트 마이크로서비스</t>
+          <t>AI agent microservices</t>
         </is>
       </c>
       <c r="E52" s="1" t="inlineStr">
@@ -2221,7 +2221,7 @@
       </c>
       <c r="D53" s="1" t="inlineStr">
         <is>
-          <t>실무용 Hono 백엔드 템플릿이자 AI 에이전트 하네스 — AI 코딩 에이전트가 아키텍처에 맞는 코드를 내도록 가이드·피드백 센서 제공</t>
+          <t>A production Hono backend template and AI agent harness - provides guides and feedback sensors so that AI coding agents produce code that fits the architecture</t>
         </is>
       </c>
       <c r="E53" s="1" t="inlineStr">
@@ -2254,7 +2254,7 @@
       </c>
       <c r="D54" s="1" t="inlineStr">
         <is>
-          <t>Easy Code(구 DeepV Code) — 주요 AI 모델과 호환되는 맞춤형 AI 코딩 어시스턴트. Claude Code·Codex 대안으로 코드 분석, 제안, 버전 롤백, 다기기 동기화, 자동 테스트 제공</t>
+          <t>Easy Code (formerly DeepV Code) - a customizable AI coding assistant compatible with major AI models. An alternative to Claude Code/Codex offering code analysis, suggestions, version rollback, multi-device sync, and automated testing</t>
         </is>
       </c>
       <c r="E54" s="1" t="inlineStr">
@@ -2287,7 +2287,7 @@
       </c>
       <c r="D55" s="1" t="inlineStr">
         <is>
-          <t>스크립트를 생성·실행해 AI 에이전트가 .NET 애플리케이션을 제어하게 하는 라이브러리</t>
+          <t>A library that lets AI agents control .NET applications by generating and running scripts</t>
         </is>
       </c>
       <c r="E55" s="1" t="inlineStr">
@@ -2320,7 +2320,7 @@
       </c>
       <c r="D56" s="1" t="inlineStr">
         <is>
-          <t>자연어로 트위터 사용하기</t>
+          <t>Using Twitter with natural language</t>
         </is>
       </c>
       <c r="E56" s="1" t="inlineStr">
@@ -2351,7 +2351,7 @@
       </c>
       <c r="D57" s="1" t="inlineStr">
         <is>
-          <t>순수 LLM 에이전트보다 최대 10배 빠른 적응형 웹 에이전트. 접근성 트리 활용, 원샷 계획</t>
+          <t>An adaptive web agent up to 10 times faster than pure LLM agents. Uses the accessibility tree, one-shot planning</t>
         </is>
       </c>
       <c r="E57" s="1" t="inlineStr">
@@ -2384,7 +2384,7 @@
       </c>
       <c r="D58" s="1" t="inlineStr">
         <is>
-          <t>FinBrain MCP 서버: FinBrain 금융 데이터셋을 AI 에이전트(Claude·VSCode 등)에 노출. 각자 API 키로 로컬 실행</t>
+          <t>FinBrain MCP server: exposes FinBrain financial datasets to AI agents (Claude, VS Code, etc.). Runs locally with each user's own API key</t>
         </is>
       </c>
       <c r="E58" s="1" t="inlineStr">
@@ -2415,7 +2415,7 @@
       </c>
       <c r="D59" s="1" t="inlineStr">
         <is>
-          <t>Planr — 제품 의도를 Codex·Claude Code·Cursor·MCP 클라이언트·사람이 공유하는 작업 그래프로 변환</t>
+          <t>Planr - turns product intent into a task graph shared by Codex, Claude Code, Cursor, MCP clients, and humans</t>
         </is>
       </c>
       <c r="E59" s="1" t="inlineStr">
@@ -2448,7 +2448,7 @@
       </c>
       <c r="D60" s="1" t="inlineStr">
         <is>
-          <t>MCP를 배우며 만든 실용 가이드·클라이언트·서버 모음(학습용)</t>
+          <t>A collection of practical guides, clients, and servers made while learning MCP (for learning)</t>
         </is>
       </c>
       <c r="E60" s="1" t="inlineStr">
@@ -2481,7 +2481,7 @@
       </c>
       <c r="D61" s="1" t="inlineStr">
         <is>
-          <t>LLM을 위한 경량·확장형 메모리 계층</t>
+          <t>A lightweight, extensible memory layer for LLMs</t>
         </is>
       </c>
       <c r="E61" s="1" t="inlineStr">
@@ -2514,7 +2514,7 @@
       </c>
       <c r="D62" s="1" t="inlineStr">
         <is>
-          <t>git 인식 CLI 할 일 관리자 + AI 에이전트 연동용 MCP 서버</t>
+          <t>A git-aware CLI to-do manager + an MCP server for AI agent integration</t>
         </is>
       </c>
       <c r="E62" s="1" t="inlineStr">
@@ -2545,7 +2545,7 @@
       </c>
       <c r="D63" s="1" t="inlineStr">
         <is>
-          <t>기업용 MCP 게이트웨이·레지스트리 — OAuth 인증, 동적 도구 탐색, 에이전트·코딩 어시스턴트 통합 접근</t>
+          <t>Enterprise MCP gateway and registry - OAuth authentication, dynamic tool discovery, unified access for agents and coding assistants</t>
         </is>
       </c>
       <c r="E63" s="1" t="inlineStr">
@@ -2578,7 +2578,7 @@
       </c>
       <c r="D64" s="1" t="inlineStr">
         <is>
-          <t>Form.io 범용 AI 에이전트 게이트웨이 — 폼 자동화용 MCP 서버</t>
+          <t>Form.io universal AI agent gateway - an MCP server for form automation</t>
         </is>
       </c>
       <c r="E64" s="1" t="inlineStr">
@@ -2611,7 +2611,7 @@
       </c>
       <c r="D65" s="1" t="inlineStr">
         <is>
-          <t>OLAF — 자연어 상호작용으로 사용자와 AI 에이전트의 교류를 돕는 단순 어시스턴트 프레임워크</t>
+          <t>OLAF - a simple assistant framework that helps users interact with AI agents through natural-language interaction</t>
         </is>
       </c>
       <c r="E65" s="1" t="inlineStr">
@@ -2644,7 +2644,7 @@
       </c>
       <c r="D66" s="1" t="inlineStr">
         <is>
-          <t>GPT·LangChain·function calling·Stable Diffusion 기반 AI 어린이 그림책 생성 앱(중국어)</t>
+          <t>An app that generates AI children's picture books, based on GPT, LangChain, function calling, and Stable Diffusion (in Chinese)</t>
         </is>
       </c>
       <c r="E66" s="1" t="inlineStr">
@@ -2675,7 +2675,7 @@
       </c>
       <c r="D67" s="1" t="inlineStr">
         <is>
-          <t>Zero Graph — AI 에이전트 프로그래밍용 미니멀 LLM 프레임워크</t>
+          <t>Zero Graph - a minimal LLM framework for programming AI agents</t>
         </is>
       </c>
       <c r="E67" s="1" t="inlineStr">
@@ -2706,7 +2706,7 @@
       </c>
       <c r="D68" s="1" t="inlineStr">
         <is>
-          <t>AI 에이전트 지식 기억에 특화된 Rust 데이터베이스 라이브러리</t>
+          <t>A Rust database library specialized for the knowledge memory of AI agents</t>
         </is>
       </c>
       <c r="E68" s="1" t="inlineStr">
@@ -2739,7 +2739,7 @@
       </c>
       <c r="D69" s="1" t="inlineStr">
         <is>
-          <t>사실 검증 기능이 있는 여행 AI 에이전트</t>
+          <t>A travel AI agent with fact-checking</t>
         </is>
       </c>
       <c r="E69" s="1" t="inlineStr">
@@ -2772,7 +2772,7 @@
       </c>
       <c r="D70" s="1" t="inlineStr">
         <is>
-          <t>보안팀용 정적 코드 분석(파일 간 오염 분석). 취약점 탐지·구조 검색, MCP 지원</t>
+          <t>Static code analysis for security teams (cross-file taint analysis). Vulnerability detection and structural search, MCP support</t>
         </is>
       </c>
       <c r="E70" s="1" t="inlineStr">
@@ -2805,7 +2805,7 @@
       </c>
       <c r="D71" s="1" t="inlineStr">
         <is>
-          <t>Home Assistant용 AI 에이전트 — 집과 대화, 자연어로 자동화 생성, 카메라 얼굴인식 분석, 이상 알림. 클라우드 또는 Ollama 로컬</t>
+          <t>An AI agent for Home Assistant - talk to your home, create automations in natural language, camera face-recognition analysis, anomaly alerts. Cloud or local via Ollama</t>
         </is>
       </c>
       <c r="E71" s="1" t="inlineStr">
@@ -2838,7 +2838,7 @@
       </c>
       <c r="D72" s="1" t="inlineStr">
         <is>
-          <t>에이전트를 위한 CLI 우선 뱅킹</t>
+          <t>CLI-first banking for agents</t>
         </is>
       </c>
       <c r="E72" s="1" t="inlineStr">
@@ -2871,7 +2871,7 @@
       </c>
       <c r="D73" s="1" t="inlineStr">
         <is>
-          <t>AI 코딩 에이전트를 위한 컨트롤 플레인</t>
+          <t>A control plane for AI coding agents</t>
         </is>
       </c>
       <c r="E73" s="1" t="inlineStr">
@@ -2904,7 +2904,7 @@
       </c>
       <c r="D74" s="1" t="inlineStr">
         <is>
-          <t>Claude 등 AI 에이전트를 아마존 셀러 파트너 API에 연결하는 최초의 MCP 클라이언트 — 재고 관리 등 판매 워크플로 자동화</t>
+          <t>The first MCP client connecting AI agents such as Claude to the Amazon Selling Partner API - automates sales workflows such as inventory management</t>
         </is>
       </c>
       <c r="E74" s="1" t="inlineStr">
@@ -2935,7 +2935,7 @@
       </c>
       <c r="D75" s="1" t="inlineStr">
         <is>
-          <t>O2.services AI Hive(AI 에이전트 동적 군집)의 사업 문서·피치 자료</t>
+          <t>Business documents and pitch materials of O2.services AI Hive (a dynamic swarm of AI agents)</t>
         </is>
       </c>
       <c r="E75" s="1" t="inlineStr">
@@ -2966,7 +2966,7 @@
       </c>
       <c r="D76" s="1" t="inlineStr">
         <is>
-          <t>AWS CDK 솔루션 청사진 라이브러리 — AI 에이전트, 문서 처리, 서버리스 등 실제 사례를 몇 분 만에 배포</t>
+          <t>AWS CDK solution blueprint library - deploy real-world cases such as AI agents, document processing, and serverless in minutes</t>
         </is>
       </c>
       <c r="E76" s="1" t="inlineStr">
@@ -2999,7 +2999,7 @@
       </c>
       <c r="D77" s="1" t="inlineStr">
         <is>
-          <t>의존성 없는 경량 워크플로 자동화 플랫폼. iPaaS·스트림 컴퓨팅·MCP·AI 기능 지원</t>
+          <t>A dependency-free lightweight workflow automation platform. Supports iPaaS, stream computing, MCP, and AI features</t>
         </is>
       </c>
       <c r="E77" s="1" t="inlineStr">
@@ -3032,7 +3032,7 @@
       </c>
       <c r="D78" s="1" t="inlineStr">
         <is>
-          <t>강의 녹취록을 자동으로 가져오는 학습 챗봇</t>
+          <t>A learning chatbot that automatically fetches lecture transcripts</t>
         </is>
       </c>
       <c r="E78" s="1" t="inlineStr">
@@ -3065,7 +3065,7 @@
       </c>
       <c r="D79" s="1" t="inlineStr">
         <is>
-          <t>올인원 LLM CLI 도구 — 셸 어시스턴트, 채팅 REPL, RAG, AI 도구·에이전트. OpenAI·Claude·Gemini·Ollama 등 지원</t>
+          <t>All-in-one LLM CLI tool - shell assistant, chat REPL, RAG, AI tools and agents. Supports OpenAI, Claude, Gemini, Ollama, and others</t>
         </is>
       </c>
       <c r="E79" s="1" t="inlineStr">
@@ -3098,7 +3098,7 @@
       </c>
       <c r="D80" s="1" t="inlineStr">
         <is>
-          <t>실무용 AI 평가·프롬프트 관리·관측 SDK. 100ms 이하 가드레일 자동 평가, 사람 개입 불필요. Python+TypeScript</t>
+          <t>SDK for production AI evaluation, prompt management, and observability. Automatic guardrail evaluation under 100 ms, no human intervention needed. Python + TypeScript</t>
         </is>
       </c>
       <c r="E80" s="1" t="inlineStr">
@@ -3131,7 +3131,7 @@
       </c>
       <c r="D81" s="1" t="inlineStr">
         <is>
-          <t>AI 에이전트들의 시스템 프롬프트를 읽기 쉽게 모아둔 것</t>
+          <t>An easy-to-read collection of the system prompts of AI agents</t>
         </is>
       </c>
       <c r="E81" s="1" t="inlineStr">
@@ -3162,7 +3162,7 @@
       </c>
       <c r="D82" s="1" t="inlineStr">
         <is>
-          <t>여러 AI 코딩 에이전트를 tmux 분할 창에서 띄우고 조율하는 세션 관리 툴킷</t>
+          <t>A session-management toolkit that launches and coordinates multiple AI coding agents in tmux split panes</t>
         </is>
       </c>
       <c r="E82" s="1" t="inlineStr">
@@ -3195,7 +3195,7 @@
       </c>
       <c r="D83" s="1" t="inlineStr">
         <is>
-          <t>OS 수준 도구로 컴퓨터를 조작하는 AI 에이전트. MCP 호환, 어떤 모델과도 작동</t>
+          <t>An AI agent that operates the computer with OS-level tools. MCP-compatible, works with any model</t>
         </is>
       </c>
       <c r="E83" s="1" t="inlineStr">
@@ -3226,7 +3226,7 @@
       </c>
       <c r="D84" s="1" t="inlineStr">
         <is>
-          <t>ALwrity — AI 우선 디지털 마케팅 플랫폼(콘텐츠 전략·생성·게시·분석·SEO·소셜 계정 관리). 진행 중</t>
+          <t>ALwrity - an AI-first digital marketing platform (content strategy, generation, publishing, analytics, SEO, social account management). Work in progress</t>
         </is>
       </c>
       <c r="E84" s="1" t="inlineStr">
@@ -3259,7 +3259,7 @@
       </c>
       <c r="D85" s="1" t="inlineStr">
         <is>
-          <t>Backlog.md — git 생태계에서 사람과 AI 에이전트의 프로젝트 협업을 관리하는 도구</t>
+          <t>Backlog.md - a tool for managing project collaboration between humans and AI agents in the git ecosystem</t>
         </is>
       </c>
       <c r="E85" s="1" t="inlineStr">
@@ -3292,7 +3292,7 @@
       </c>
       <c r="D86" s="1" t="inlineStr">
         <is>
-          <t>말로 쓰는 상시 가동 '세컨드 브레인'. 텔레그램 음성 메모 → Obsidian 보관함에 정리·링크. Claude 구독으로 24시간 실행</t>
+          <t>An always-on voice-driven 'second brain'. Telegram voice memos -&gt; organized and linked in an Obsidian vault. Runs 24 hours on a Claude subscription</t>
         </is>
       </c>
       <c r="E86" s="1" t="inlineStr">
@@ -3325,7 +3325,7 @@
       </c>
       <c r="D87" s="1" t="inlineStr">
         <is>
-          <t>Org-mode의 ai 블록에서 LLM과 AI 에이전트 호출</t>
+          <t>Calling LLMs and AI agents from ai blocks in Org-mode</t>
         </is>
       </c>
       <c r="E87" s="1" t="inlineStr">
@@ -3358,7 +3358,7 @@
       </c>
       <c r="D88" s="1" t="inlineStr">
         <is>
-          <t>가장 싼 가격으로 여행하도록 돕는 AI 에이전트</t>
+          <t>An AI agent that helps you travel at the lowest price</t>
         </is>
       </c>
       <c r="E88" s="1" t="inlineStr">
@@ -3389,7 +3389,7 @@
       </c>
       <c r="D89" s="1" t="inlineStr">
         <is>
-          <t>vvaifu.fun 클론(포크): AI 크립토 에이전트 + 솔라나 스마트 컨트랙트 소스</t>
+          <t>A clone (fork) of vvaifu.fun: AI crypto agent + Solana smart-contract source</t>
         </is>
       </c>
       <c r="E89" s="1" t="inlineStr">
@@ -3422,7 +3422,7 @@
       </c>
       <c r="D90" s="1" t="inlineStr">
         <is>
-          <t>DSPy용 Claude Code — DSPy 코드 최적화 CLI, AI 기반 DSPy 개발 어시스턴트</t>
+          <t>Claude Code for DSPy - a CLI for optimizing DSPy code, an AI-powered DSPy development assistant</t>
         </is>
       </c>
       <c r="E90" s="1" t="inlineStr">
@@ -3455,7 +3455,7 @@
       </c>
       <c r="D91" s="1" t="inlineStr">
         <is>
-          <t>Alchemy 공식 MCP 서버. AI 에이전트가 Alchemy 블록체인 API와 상호작용</t>
+          <t>Official Alchemy MCP server. AI agents interact with the Alchemy blockchain APIs</t>
         </is>
       </c>
       <c r="E91" s="1" t="inlineStr">
@@ -3486,7 +3486,7 @@
       </c>
       <c r="D92" s="1" t="inlineStr">
         <is>
-          <t>KogniSwarm — GPT-4로 자율 AI 애플리케이션을 개발하는 Kotlin 오픈소스 프로젝트</t>
+          <t>KogniSwarm - an open-source Kotlin project for developing autonomous AI applications with GPT-4</t>
         </is>
       </c>
       <c r="E92" s="1" t="inlineStr">
@@ -3519,7 +3519,7 @@
       </c>
       <c r="D93" s="1" t="inlineStr">
         <is>
-          <t>Godot에서 Copilot을 쓰기 위한 마크다운 가이드라인(코딩 표준·워크플로 규칙)</t>
+          <t>Markdown guidelines for using Copilot in Godot (coding standards, workflow rules)</t>
         </is>
       </c>
       <c r="E93" s="1" t="inlineStr">
@@ -3552,7 +3552,7 @@
       </c>
       <c r="D94" s="1" t="inlineStr">
         <is>
-          <t>LLM 에이전트로 실험을 돌리기 위한 oTree 앱 템플릿 모음</t>
+          <t>A collection of oTree app templates for running experiments with LLM agents</t>
         </is>
       </c>
       <c r="E94" s="1" t="inlineStr">
@@ -3583,7 +3583,7 @@
       </c>
       <c r="D95" s="1" t="inlineStr">
         <is>
-          <t>SIGIR 2024 논문: TRAD — 단계별 사고 검색과 정렬된 의사결정으로 LLM 에이전트 강화</t>
+          <t>SIGIR 2024 paper: TRAD - enhancing LLM agents with step-wise thought retrieval and aligned decision making</t>
         </is>
       </c>
       <c r="E95" s="1" t="inlineStr">
@@ -3614,7 +3614,7 @@
       </c>
       <c r="D96" s="1" t="inlineStr">
         <is>
-          <t>⚠️ 폐기됨(DEPRECATED) — coderag로 대체</t>
+          <t>⚠️ DEPRECATED - replaced by coderag</t>
         </is>
       </c>
       <c r="E96" s="1" t="inlineStr">
@@ -3647,7 +3647,7 @@
       </c>
       <c r="D97" s="1" t="inlineStr">
         <is>
-          <t>Claude Code 강화 컴포넌트 109개 — 에이전트 22, 명령 32, 스킬 55, 플러그인 13. 자율 개발 루프·DDD·git 자동화 등</t>
+          <t>109 components that enhance Claude Code - 22 agents, 32 commands, 55 skills, 13 plugins. Autonomous development loop, DDD, git automation, etc.</t>
         </is>
       </c>
       <c r="E97" s="1" t="inlineStr">
@@ -3680,7 +3680,7 @@
       </c>
       <c r="D98" s="1" t="inlineStr">
         <is>
-          <t>(설명 없음)</t>
+          <t>(no description)</t>
         </is>
       </c>
       <c r="E98" s="1" t="n">
@@ -3711,7 +3711,7 @@
       </c>
       <c r="D99" s="1" t="inlineStr">
         <is>
-          <t>사람 개입(HITL) 안전장치 옵션, MCP 연동, 테마 지원 CLI 출력을 갖춘 AI 에이전트</t>
+          <t>An AI agent with optional human-in-the-loop (HITL) safeguards, MCP integration, and themed CLI output</t>
         </is>
       </c>
       <c r="E99" s="1" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="D100" s="1" t="inlineStr">
         <is>
-          <t>AgentKit으로 AI 에이전트를 Chargebee(구독 결제)와 연동해 청구·구독 워크플로 자동화</t>
+          <t>Automating billing and subscription workflows by connecting AI agents to Chargebee (subscription billing) with AgentKit</t>
         </is>
       </c>
       <c r="E100" s="1" t="inlineStr">
@@ -3777,7 +3777,7 @@
       </c>
       <c r="D101" s="1" t="inlineStr">
         <is>
-          <t>ICLR 2026 논문 공개 코드: 다중 턴 상호작용으로 LLM 에이전트 기억 평가</t>
+          <t>Released code of an ICLR 2026 paper: evaluating the memory of LLM agents through multi-turn interactions</t>
         </is>
       </c>
       <c r="E101" s="1" t="inlineStr">
@@ -3810,7 +3810,7 @@
       </c>
       <c r="D102" s="1" t="inlineStr">
         <is>
-          <t>AI 에이전트 실행 추적에서 출처·감사 기록 추출</t>
+          <t>Extracting provenance and audit records from AI agent execution traces</t>
         </is>
       </c>
       <c r="E102" s="1" t="inlineStr">
@@ -3843,7 +3843,7 @@
       </c>
       <c r="D103" s="1" t="inlineStr">
         <is>
-          <t>Ecma TC-56 NLIP(자연어 상호작용 프로토콜) 관련 문서 저장소</t>
+          <t>A documentation repository for Ecma TC-56 NLIP (Natural Language Interaction Protocol)</t>
         </is>
       </c>
       <c r="E103" s="1" t="inlineStr">
@@ -3876,7 +3876,7 @@
       </c>
       <c r="D104" s="1" t="inlineStr">
         <is>
-          <t>Vercel AI SDK 기반 임베드형 에이전트 AI 채팅</t>
+          <t>Embeddable agentic AI chat based on the Vercel AI SDK</t>
         </is>
       </c>
       <c r="E104" s="1" t="inlineStr">
@@ -3909,7 +3909,7 @@
       </c>
       <c r="D105" s="1" t="inlineStr">
         <is>
-          <t>ManusMCP — Flowise로 AI 에이전트 워크플로 구현. 플래너·파일마법사·명령실행·웹탐색 역할별 에이전트</t>
+          <t>ManusMCP - AI agent workflows implemented with Flowise. Role-specific agents: planner, file wizard, command executor, web explorer</t>
         </is>
       </c>
       <c r="E105" s="1" t="inlineStr">
@@ -3940,7 +3940,7 @@
       </c>
       <c r="D106" s="1" t="inlineStr">
         <is>
-          <t>Google ADK·Gemini·A2UI 기반 AI 기술면접관. 적응형 면접·학습 안내·코드 분석 멀티에이전트 시스템</t>
+          <t>An AI technical interviewer based on Google ADK, Gemini, and A2UI. A multi-agent system for adaptive interviews, learning guidance, and code analysis</t>
         </is>
       </c>
       <c r="E106" s="1" t="inlineStr">
@@ -3973,7 +3973,7 @@
       </c>
       <c r="D107" s="1" t="inlineStr">
         <is>
-          <t>AI 에이전트를 위한 셸 초능력(Shell Superpowers)</t>
+          <t>Shell superpowers for AI agents</t>
         </is>
       </c>
       <c r="E107" s="1" t="inlineStr">
@@ -4006,7 +4006,7 @@
       </c>
       <c r="D108" s="1" t="inlineStr">
         <is>
-          <t>BRAD — 생물정보학용 LLM 기반 검색증강 디지털 어시스턴트 에이전트</t>
+          <t>BRAD - an LLM-based retrieval-augmented digital assistant agent for bioinformatics</t>
         </is>
       </c>
       <c r="E108" s="1" t="inlineStr">
@@ -4039,7 +4039,7 @@
       </c>
       <c r="D109" s="1" t="inlineStr">
         <is>
-          <t>Dremio(데이터 레이크하우스) MCP 서버</t>
+          <t>Dremio (data lakehouse) MCP server</t>
         </is>
       </c>
       <c r="E109" s="1" t="inlineStr">
@@ -4072,7 +4072,7 @@
       </c>
       <c r="D110" s="1" t="inlineStr">
         <is>
-          <t>실무 AI 앱용 오픈 Python 에이전트 하네스 — 도구·MCP·메모리·작업공간·텔레메트리·서브에이전트·백그라운드 작업</t>
+          <t>An open Python agent harness for production AI apps - tools, MCP, memory, workspace, telemetry, sub-agents, background tasks</t>
         </is>
       </c>
       <c r="E110" s="1" t="inlineStr">
@@ -4105,7 +4105,7 @@
       </c>
       <c r="D111" s="1" t="inlineStr">
         <is>
-          <t>Laravel용 AI 에이전트 프레임워크</t>
+          <t>An AI agent framework for Laravel</t>
         </is>
       </c>
       <c r="E111" s="1" t="inlineStr">
@@ -4136,7 +4136,7 @@
       </c>
       <c r="D112" s="1" t="inlineStr">
         <is>
-          <t>MCP-Zero: 자율 LLM 에이전트를 위한 능동적 도구 탐색(논문)</t>
+          <t>MCP-Zero: active tool discovery for autonomous LLM agents (paper)</t>
         </is>
       </c>
       <c r="E112" s="1" t="inlineStr">
@@ -4167,7 +4167,7 @@
       </c>
       <c r="D113" s="1" t="inlineStr">
         <is>
-          <t>AGI 프레임워크·소프트웨어·자료 정리 목록(awesome 리스트)</t>
+          <t>A curated list of AGI frameworks, software, and resources (awesome list)</t>
         </is>
       </c>
       <c r="E113" s="1" t="inlineStr">
@@ -4200,7 +4200,7 @@
       </c>
       <c r="D114" s="1" t="inlineStr">
         <is>
-          <t>논문 코드·데이터 공개 — DelTA: 다층 메모리 기반 온라인 문서 단위 번역 에이전트</t>
+          <t>Release of paper code and data - DelTA: an online document-level translation agent based on multi-level memory</t>
         </is>
       </c>
       <c r="E114" s="1" t="inlineStr">
@@ -4233,7 +4233,7 @@
       </c>
       <c r="D115" s="1" t="inlineStr">
         <is>
-          <t>소프트웨어 엔지니어를 위한 AI 에이전트 오픈 북(포르투갈어). Python·LangChain·LangGraph·RAG·로컬/원격 모델</t>
+          <t>An open book on AI agents for software engineers (in Portuguese). Python, LangChain, LangGraph, RAG, local/remote models</t>
         </is>
       </c>
       <c r="E115" s="1" t="inlineStr">
@@ -4266,7 +4266,7 @@
       </c>
       <c r="D116" s="1" t="inlineStr">
         <is>
-          <t>Claude Code 등 MCP 클라이언트용 범용 MCP 서버 — PowerShell 모듈 1만 개 이상과 모든 CLI 도구에 AI 접근</t>
+          <t>A universal MCP server for MCP clients such as Claude Code - AI access to more than 10,000 PowerShell modules and every CLI tool</t>
         </is>
       </c>
       <c r="E116" s="1" t="inlineStr">
@@ -4299,7 +4299,7 @@
       </c>
       <c r="D117" s="1" t="inlineStr">
         <is>
-          <t>Ruby AI 에이전트 SDK — OpenAI Agents SDK에서 영감</t>
+          <t>A Ruby AI agent SDK - inspired by the OpenAI Agents SDK</t>
         </is>
       </c>
       <c r="E117" s="1" t="inlineStr">
@@ -4332,7 +4332,7 @@
       </c>
       <c r="D118" s="1" t="inlineStr">
         <is>
-          <t>개인화 AI 에이전트를 가장 빠르게 만드는 방법</t>
+          <t>The fastest way to build personalized AI agents</t>
         </is>
       </c>
       <c r="E118" s="1" t="inlineStr">
@@ -4365,7 +4365,7 @@
       </c>
       <c r="D119" s="1" t="inlineStr">
         <is>
-          <t>GitHub 리포지토리를 긁어 AI로 분석한 뒤 관심 있을 프로젝트를 디스코드 웹훅으로 보내주는 프로젝트</t>
+          <t>A project that scrapes GitHub repositories, analyzes them with AI, and sends projects of likely interest via a Discord webhook</t>
         </is>
       </c>
       <c r="E119" s="1" t="inlineStr">
@@ -4398,7 +4398,7 @@
       </c>
       <c r="D120" s="1" t="inlineStr">
         <is>
-          <t>MiniMax M3 기반 Cursor 규칙 모음 — 명확화 우선 프롬프팅, 도구 오케스트레이션으로 실무용 AI 코딩</t>
+          <t>A collection of Cursor rules based on MiniMax M3 - clarification-first prompting and tool orchestration for production AI coding</t>
         </is>
       </c>
       <c r="E120" s="1" t="inlineStr">
@@ -4431,7 +4431,7 @@
       </c>
       <c r="D121" s="1" t="inlineStr">
         <is>
-          <t>codebadger — Joern 코드 속성 그래프로 코드베이스 구조와 데이터 흐름을 AI 에이전트가 조회할 수 있게 해주는 컨테이너형 MCP 서버</t>
+          <t>codebadger - a containerized MCP server that lets AI agents query codebase structure and data flow through Joern code property graphs</t>
         </is>
       </c>
       <c r="E121" s="1" t="inlineStr">
@@ -4485,7 +4485,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>번호</t>
+          <t>item_no</t>
         </is>
       </c>
       <c r="B1" s="2" t="inlineStr">
@@ -4495,17 +4495,17 @@
       </c>
       <c r="C1" s="2" t="inlineStr">
         <is>
-          <t>링크</t>
+          <t>Link</t>
         </is>
       </c>
       <c r="D1" s="2" t="inlineStr">
         <is>
-          <t>한글 설명</t>
+          <t>Short description</t>
         </is>
       </c>
       <c r="E1" s="2" t="inlineStr">
         <is>
-          <t>description (원문)</t>
+          <t>description (original)</t>
         </is>
       </c>
       <c r="F1" s="2" t="inlineStr">
@@ -4515,37 +4515,37 @@
       </c>
       <c r="G1" s="2" t="inlineStr">
         <is>
-          <t>A 원판정</t>
+          <t>A original judgment</t>
         </is>
       </c>
       <c r="H1" s="2" t="inlineStr">
         <is>
-          <t>B 원판정</t>
+          <t>B original judgment</t>
         </is>
       </c>
       <c r="I1" s="2" t="inlineStr">
         <is>
-          <t>C 원판정</t>
+          <t>C original judgment</t>
         </is>
       </c>
       <c r="J1" s="2" t="inlineStr">
         <is>
-          <t>찬성 수</t>
+          <t>Votes for agent</t>
         </is>
       </c>
       <c r="K1" s="2" t="inlineStr">
         <is>
-          <t>판정(1/2/3)</t>
+          <t>Judgment (1/2/3)</t>
         </is>
       </c>
       <c r="L1" s="2" t="inlineStr">
         <is>
-          <t>규칙 번호</t>
+          <t>Rule no.</t>
         </is>
       </c>
       <c r="M1" s="2" t="inlineStr">
         <is>
-          <t>메모</t>
+          <t>Notes</t>
         </is>
       </c>
     </row>
@@ -4565,7 +4565,7 @@
       </c>
       <c r="D2" s="1" t="inlineStr">
         <is>
-          <t>Dremio(데이터 레이크하우스) MCP 서버</t>
+          <t>Dremio (data lakehouse) MCP server</t>
         </is>
       </c>
       <c r="E2" s="1" t="inlineStr">
@@ -4580,17 +4580,17 @@
       </c>
       <c r="G2" s="1" t="inlineStr">
         <is>
-          <t>3 무관·판정불가</t>
+          <t>3 Unrelated/undecidable</t>
         </is>
       </c>
       <c r="H2" s="1" t="inlineStr">
         <is>
-          <t>1 에이전트 소프트웨어</t>
+          <t>1 Agent software</t>
         </is>
       </c>
       <c r="I2" s="1" t="inlineStr">
         <is>
-          <t>1 에이전트 소프트웨어</t>
+          <t>1 Agent software</t>
         </is>
       </c>
       <c r="J2" s="1" t="n">
@@ -4616,7 +4616,7 @@
       </c>
       <c r="D3" s="1" t="inlineStr">
         <is>
-          <t>PydanticAI와 Permit.io 세밀 권한 프레임워크로 안전한 AI 에이전트를 구현하는 시연(데모)</t>
+          <t>A demonstration (demo) of building secure AI agents with PydanticAI and the Permit.io fine-grained authorization framework</t>
         </is>
       </c>
       <c r="E3" s="1" t="inlineStr">
@@ -4631,17 +4631,17 @@
       </c>
       <c r="G3" s="1" t="inlineStr">
         <is>
-          <t>1 에이전트 소프트웨어</t>
+          <t>1 Agent software</t>
         </is>
       </c>
       <c r="H3" s="1" t="inlineStr">
         <is>
-          <t>2 학습·참고 자료</t>
+          <t>2 Learning/reference resource</t>
         </is>
       </c>
       <c r="I3" s="1" t="inlineStr">
         <is>
-          <t>2 학습·참고 자료</t>
+          <t>2 Learning/reference resource</t>
         </is>
       </c>
       <c r="J3" s="1" t="n">
@@ -4667,7 +4667,7 @@
       </c>
       <c r="D4" s="1" t="inlineStr">
         <is>
-          <t>MiniMax M3 기반 Cursor 규칙 모음 — 명확화 우선 프롬프팅, 도구 오케스트레이션으로 실무용 AI 코딩</t>
+          <t>A collection of Cursor rules based on MiniMax M3 - clarification-first prompting and tool orchestration for production AI coding</t>
         </is>
       </c>
       <c r="E4" s="1" t="inlineStr">
@@ -4682,17 +4682,17 @@
       </c>
       <c r="G4" s="1" t="inlineStr">
         <is>
-          <t>1 에이전트 소프트웨어</t>
+          <t>1 Agent software</t>
         </is>
       </c>
       <c r="H4" s="1" t="inlineStr">
         <is>
-          <t>3 무관·판정불가</t>
+          <t>3 Unrelated/undecidable</t>
         </is>
       </c>
       <c r="I4" s="1" t="inlineStr">
         <is>
-          <t>1 에이전트 소프트웨어</t>
+          <t>1 Agent software</t>
         </is>
       </c>
       <c r="J4" s="1" t="n">
@@ -4718,7 +4718,7 @@
       </c>
       <c r="D5" s="1" t="inlineStr">
         <is>
-          <t>실무용 AI 평가·프롬프트 관리·관측 SDK. 100ms 이하 가드레일 자동 평가, 사람 개입 불필요. Python+TypeScript</t>
+          <t>SDK for production AI evaluation, prompt management, and observability. Automatic guardrail evaluation under 100 ms, no human intervention needed. Python + TypeScript</t>
         </is>
       </c>
       <c r="E5" s="1" t="inlineStr">
@@ -4733,17 +4733,17 @@
       </c>
       <c r="G5" s="1" t="inlineStr">
         <is>
-          <t>1 에이전트 소프트웨어</t>
+          <t>1 Agent software</t>
         </is>
       </c>
       <c r="H5" s="1" t="inlineStr">
         <is>
-          <t>3 무관·판정불가</t>
+          <t>3 Unrelated/undecidable</t>
         </is>
       </c>
       <c r="I5" s="1" t="inlineStr">
         <is>
-          <t>1 에이전트 소프트웨어</t>
+          <t>1 Agent software</t>
         </is>
       </c>
       <c r="J5" s="1" t="n">
@@ -4769,7 +4769,7 @@
       </c>
       <c r="D6" s="1" t="inlineStr">
         <is>
-          <t>PHP 프로젝트용 에이전트 스킬 배포·관리 Composer 플러그인</t>
+          <t>A Composer plugin for distributing and managing agent skills for PHP projects</t>
         </is>
       </c>
       <c r="E6" s="1" t="inlineStr">
@@ -4784,17 +4784,17 @@
       </c>
       <c r="G6" s="1" t="inlineStr">
         <is>
-          <t>3 무관·판정불가</t>
+          <t>3 Unrelated/undecidable</t>
         </is>
       </c>
       <c r="H6" s="1" t="inlineStr">
         <is>
-          <t>1 에이전트 소프트웨어</t>
+          <t>1 Agent software</t>
         </is>
       </c>
       <c r="I6" s="1" t="inlineStr">
         <is>
-          <t>1 에이전트 소프트웨어</t>
+          <t>1 Agent software</t>
         </is>
       </c>
       <c r="J6" s="1" t="n">
@@ -4820,7 +4820,7 @@
       </c>
       <c r="D7" s="1" t="inlineStr">
         <is>
-          <t>AI 에이전트·MCP·AI 워크플로 자동화 모음(AI 에이전트용 MCP 서버 약 400개)</t>
+          <t>A collection of AI agents, MCP, and AI workflow automation (about 400 MCP servers for AI agents)</t>
         </is>
       </c>
       <c r="E7" s="1" t="inlineStr">
@@ -4835,17 +4835,17 @@
       </c>
       <c r="G7" s="1" t="inlineStr">
         <is>
-          <t>1 에이전트 소프트웨어</t>
+          <t>1 Agent software</t>
         </is>
       </c>
       <c r="H7" s="1" t="inlineStr">
         <is>
-          <t>3 무관·판정불가</t>
+          <t>3 Unrelated/undecidable</t>
         </is>
       </c>
       <c r="I7" s="1" t="inlineStr">
         <is>
-          <t>2 학습·참고 자료</t>
+          <t>2 Learning/reference resource</t>
         </is>
       </c>
       <c r="J7" s="1" t="n">
@@ -4871,7 +4871,7 @@
       </c>
       <c r="D8" s="1" t="inlineStr">
         <is>
-          <t>LLM 에이전트로 실험을 돌리기 위한 oTree 앱 템플릿 모음</t>
+          <t>A collection of oTree app templates for running experiments with LLM agents</t>
         </is>
       </c>
       <c r="E8" s="1" t="inlineStr">
@@ -4884,17 +4884,17 @@
       </c>
       <c r="G8" s="1" t="inlineStr">
         <is>
-          <t>1 에이전트 소프트웨어</t>
+          <t>1 Agent software</t>
         </is>
       </c>
       <c r="H8" s="1" t="inlineStr">
         <is>
-          <t>3 무관·판정불가</t>
+          <t>3 Unrelated/undecidable</t>
         </is>
       </c>
       <c r="I8" s="1" t="inlineStr">
         <is>
-          <t>2 학습·참고 자료</t>
+          <t>2 Learning/reference resource</t>
         </is>
       </c>
       <c r="J8" s="1" t="n">
@@ -4920,7 +4920,7 @@
       </c>
       <c r="D9" s="1" t="inlineStr">
         <is>
-          <t>devcontainer.json 설정으로 개발 컨테이너를 생성·구성하는 MCP 서버</t>
+          <t>An MCP server that creates and configures development containers from devcontainer.json settings</t>
         </is>
       </c>
       <c r="E9" s="1" t="inlineStr">
@@ -4935,17 +4935,17 @@
       </c>
       <c r="G9" s="1" t="inlineStr">
         <is>
-          <t>3 무관·판정불가</t>
+          <t>3 Unrelated/undecidable</t>
         </is>
       </c>
       <c r="H9" s="1" t="inlineStr">
         <is>
-          <t>1 에이전트 소프트웨어</t>
+          <t>1 Agent software</t>
         </is>
       </c>
       <c r="I9" s="1" t="inlineStr">
         <is>
-          <t>1 에이전트 소프트웨어</t>
+          <t>1 Agent software</t>
         </is>
       </c>
       <c r="J9" s="1" t="n">
@@ -4971,7 +4971,7 @@
       </c>
       <c r="D10" s="1" t="inlineStr">
         <is>
-          <t>ICLR 2026 논문: Agent-X — 시각 중심 에이전트 과제의 멀티모달 추론 평가</t>
+          <t>ICLR 2026 paper: Agent-X - evaluating multimodal reasoning on vision-centric agent tasks</t>
         </is>
       </c>
       <c r="E10" s="1" t="inlineStr">
@@ -4986,17 +4986,17 @@
       </c>
       <c r="G10" s="1" t="inlineStr">
         <is>
-          <t>1 에이전트 소프트웨어</t>
+          <t>1 Agent software</t>
         </is>
       </c>
       <c r="H10" s="1" t="inlineStr">
         <is>
-          <t>2 학습·참고 자료</t>
+          <t>2 Learning/reference resource</t>
         </is>
       </c>
       <c r="I10" s="1" t="inlineStr">
         <is>
-          <t>2 학습·참고 자료</t>
+          <t>2 Learning/reference resource</t>
         </is>
       </c>
       <c r="J10" s="1" t="n">
@@ -5022,7 +5022,7 @@
       </c>
       <c r="D11" s="1" t="inlineStr">
         <is>
-          <t>ICLR 2026 논문 공개 코드: 다중 턴 상호작용으로 LLM 에이전트 기억 평가</t>
+          <t>Released code of an ICLR 2026 paper: evaluating the memory of LLM agents through multi-turn interactions</t>
         </is>
       </c>
       <c r="E11" s="1" t="inlineStr">
@@ -5037,17 +5037,17 @@
       </c>
       <c r="G11" s="1" t="inlineStr">
         <is>
-          <t>1 에이전트 소프트웨어</t>
+          <t>1 Agent software</t>
         </is>
       </c>
       <c r="H11" s="1" t="inlineStr">
         <is>
-          <t>2 학습·참고 자료</t>
+          <t>2 Learning/reference resource</t>
         </is>
       </c>
       <c r="I11" s="1" t="inlineStr">
         <is>
-          <t>2 학습·참고 자료</t>
+          <t>2 Learning/reference resource</t>
         </is>
       </c>
       <c r="J11" s="1" t="n">
@@ -5073,7 +5073,7 @@
       </c>
       <c r="D12" s="1" t="inlineStr">
         <is>
-          <t>보안팀용 정적 코드 분석(파일 간 오염 분석). 취약점 탐지·구조 검색, MCP 지원</t>
+          <t>Static code analysis for security teams (cross-file taint analysis). Vulnerability detection and structural search, MCP support</t>
         </is>
       </c>
       <c r="E12" s="1" t="inlineStr">
@@ -5088,17 +5088,17 @@
       </c>
       <c r="G12" s="1" t="inlineStr">
         <is>
-          <t>3 무관·판정불가</t>
+          <t>3 Unrelated/undecidable</t>
         </is>
       </c>
       <c r="H12" s="1" t="inlineStr">
         <is>
-          <t>1 에이전트 소프트웨어</t>
+          <t>1 Agent software</t>
         </is>
       </c>
       <c r="I12" s="1" t="inlineStr">
         <is>
-          <t>1 에이전트 소프트웨어</t>
+          <t>1 Agent software</t>
         </is>
       </c>
       <c r="J12" s="1" t="n">
@@ -5124,7 +5124,7 @@
       </c>
       <c r="D13" s="1" t="inlineStr">
         <is>
-          <t>GitHub 리포지토리를 긁어 AI로 분석한 뒤 관심 있을 프로젝트를 디스코드 웹훅으로 보내주는 프로젝트</t>
+          <t>A project that scrapes GitHub repositories, analyzes them with AI, and sends projects of likely interest via a Discord webhook</t>
         </is>
       </c>
       <c r="E13" s="1" t="inlineStr">
@@ -5139,17 +5139,17 @@
       </c>
       <c r="G13" s="1" t="inlineStr">
         <is>
-          <t>3 무관·판정불가</t>
+          <t>3 Unrelated/undecidable</t>
         </is>
       </c>
       <c r="H13" s="1" t="inlineStr">
         <is>
-          <t>1 에이전트 소프트웨어</t>
+          <t>1 Agent software</t>
         </is>
       </c>
       <c r="I13" s="1" t="inlineStr">
         <is>
-          <t>1 에이전트 소프트웨어</t>
+          <t>1 Agent software</t>
         </is>
       </c>
       <c r="J13" s="1" t="n">
@@ -5175,7 +5175,7 @@
       </c>
       <c r="D14" s="1" t="inlineStr">
         <is>
-          <t>논문 코드·데이터 공개 — DelTA: 다층 메모리 기반 온라인 문서 단위 번역 에이전트</t>
+          <t>Release of paper code and data - DelTA: an online document-level translation agent based on multi-level memory</t>
         </is>
       </c>
       <c r="E14" s="1" t="inlineStr">
@@ -5190,17 +5190,17 @@
       </c>
       <c r="G14" s="1" t="inlineStr">
         <is>
-          <t>1 에이전트 소프트웨어</t>
+          <t>1 Agent software</t>
         </is>
       </c>
       <c r="H14" s="1" t="inlineStr">
         <is>
-          <t>2 학습·참고 자료</t>
+          <t>2 Learning/reference resource</t>
         </is>
       </c>
       <c r="I14" s="1" t="inlineStr">
         <is>
-          <t>2 학습·참고 자료</t>
+          <t>2 Learning/reference resource</t>
         </is>
       </c>
       <c r="J14" s="1" t="n">
@@ -5226,7 +5226,7 @@
       </c>
       <c r="D15" s="1" t="inlineStr">
         <is>
-          <t>소프트웨어 엔지니어를 위한 AI 에이전트 오픈 북(포르투갈어). Python·LangChain·LangGraph·RAG·로컬/원격 모델</t>
+          <t>An open book on AI agents for software engineers (in Portuguese). Python, LangChain, LangGraph, RAG, local/remote models</t>
         </is>
       </c>
       <c r="E15" s="1" t="inlineStr">
@@ -5241,17 +5241,17 @@
       </c>
       <c r="G15" s="1" t="inlineStr">
         <is>
-          <t>1 에이전트 소프트웨어</t>
+          <t>1 Agent software</t>
         </is>
       </c>
       <c r="H15" s="1" t="inlineStr">
         <is>
-          <t>2 학습·참고 자료</t>
+          <t>2 Learning/reference resource</t>
         </is>
       </c>
       <c r="I15" s="1" t="inlineStr">
         <is>
-          <t>2 학습·참고 자료</t>
+          <t>2 Learning/reference resource</t>
         </is>
       </c>
       <c r="J15" s="1" t="n">
@@ -5277,7 +5277,7 @@
       </c>
       <c r="D16" s="1" t="inlineStr">
         <is>
-          <t>AWS CDK 솔루션 청사진 라이브러리 — AI 에이전트, 문서 처리, 서버리스 등 실제 사례를 몇 분 만에 배포</t>
+          <t>AWS CDK solution blueprint library - deploy real-world cases such as AI agents, document processing, and serverless in minutes</t>
         </is>
       </c>
       <c r="E16" s="1" t="inlineStr">
@@ -5292,17 +5292,17 @@
       </c>
       <c r="G16" s="1" t="inlineStr">
         <is>
-          <t>1 에이전트 소프트웨어</t>
+          <t>1 Agent software</t>
         </is>
       </c>
       <c r="H16" s="1" t="inlineStr">
         <is>
-          <t>3 무관·판정불가</t>
+          <t>3 Unrelated/undecidable</t>
         </is>
       </c>
       <c r="I16" s="1" t="inlineStr">
         <is>
-          <t>1 에이전트 소프트웨어</t>
+          <t>1 Agent software</t>
         </is>
       </c>
       <c r="J16" s="1" t="n">
@@ -5328,7 +5328,7 @@
       </c>
       <c r="D17" s="1" t="inlineStr">
         <is>
-          <t>AI 에이전트들의 시스템 프롬프트를 읽기 쉽게 모아둔 것</t>
+          <t>An easy-to-read collection of the system prompts of AI agents</t>
         </is>
       </c>
       <c r="E17" s="1" t="inlineStr">
@@ -5341,17 +5341,17 @@
       </c>
       <c r="G17" s="1" t="inlineStr">
         <is>
-          <t>1 에이전트 소프트웨어</t>
+          <t>1 Agent software</t>
         </is>
       </c>
       <c r="H17" s="1" t="inlineStr">
         <is>
-          <t>2 학습·참고 자료</t>
+          <t>2 Learning/reference resource</t>
         </is>
       </c>
       <c r="I17" s="1" t="inlineStr">
         <is>
-          <t>2 학습·참고 자료</t>
+          <t>2 Learning/reference resource</t>
         </is>
       </c>
       <c r="J17" s="1" t="n">
@@ -5377,7 +5377,7 @@
       </c>
       <c r="D18" s="1" t="inlineStr">
         <is>
-          <t>(설명 없음)</t>
+          <t>(no description)</t>
         </is>
       </c>
       <c r="E18" s="1" t="n">
@@ -5390,17 +5390,17 @@
       </c>
       <c r="G18" s="1" t="inlineStr">
         <is>
-          <t>3 무관·판정불가</t>
+          <t>3 Unrelated/undecidable</t>
         </is>
       </c>
       <c r="H18" s="1" t="inlineStr">
         <is>
-          <t>3 무관·판정불가</t>
+          <t>3 Unrelated/undecidable</t>
         </is>
       </c>
       <c r="I18" s="1" t="inlineStr">
         <is>
-          <t>1 에이전트 소프트웨어</t>
+          <t>1 Agent software</t>
         </is>
       </c>
       <c r="J18" s="1" t="n">
@@ -5426,7 +5426,7 @@
       </c>
       <c r="D19" s="1" t="inlineStr">
         <is>
-          <t>Simli WebRTC AI 에이전트 데모</t>
+          <t>Simli WebRTC AI agent demo</t>
         </is>
       </c>
       <c r="E19" s="1" t="inlineStr">
@@ -5439,17 +5439,17 @@
       </c>
       <c r="G19" s="1" t="inlineStr">
         <is>
-          <t>1 에이전트 소프트웨어</t>
+          <t>1 Agent software</t>
         </is>
       </c>
       <c r="H19" s="1" t="inlineStr">
         <is>
-          <t>3 무관·판정불가</t>
+          <t>3 Unrelated/undecidable</t>
         </is>
       </c>
       <c r="I19" s="1" t="inlineStr">
         <is>
-          <t>2 학습·참고 자료</t>
+          <t>2 Learning/reference resource</t>
         </is>
       </c>
       <c r="J19" s="1" t="n">
@@ -5475,7 +5475,7 @@
       </c>
       <c r="D20" s="1" t="inlineStr">
         <is>
-          <t>LLM 파이프라인과 AI 에이전트</t>
+          <t>LLM pipelines and AI agents</t>
         </is>
       </c>
       <c r="E20" s="1" t="inlineStr">
@@ -5488,17 +5488,17 @@
       </c>
       <c r="G20" s="1" t="inlineStr">
         <is>
-          <t>1 에이전트 소프트웨어</t>
+          <t>1 Agent software</t>
         </is>
       </c>
       <c r="H20" s="1" t="inlineStr">
         <is>
-          <t>3 무관·판정불가</t>
+          <t>3 Unrelated/undecidable</t>
         </is>
       </c>
       <c r="I20" s="1" t="inlineStr">
         <is>
-          <t>1 에이전트 소프트웨어</t>
+          <t>1 Agent software</t>
         </is>
       </c>
       <c r="J20" s="1" t="n">
@@ -5524,7 +5524,7 @@
       </c>
       <c r="D21" s="1" t="inlineStr">
         <is>
-          <t>논문 코드: 팝업으로 비전-언어 컴퓨터 에이전트를 공격하기</t>
+          <t>Paper code: attacking vision-language computer agents with pop-ups</t>
         </is>
       </c>
       <c r="E21" s="1" t="inlineStr">
@@ -5539,17 +5539,17 @@
       </c>
       <c r="G21" s="1" t="inlineStr">
         <is>
-          <t>1 에이전트 소프트웨어</t>
+          <t>1 Agent software</t>
         </is>
       </c>
       <c r="H21" s="1" t="inlineStr">
         <is>
-          <t>2 학습·참고 자료</t>
+          <t>2 Learning/reference resource</t>
         </is>
       </c>
       <c r="I21" s="1" t="inlineStr">
         <is>
-          <t>2 학습·참고 자료</t>
+          <t>2 Learning/reference resource</t>
         </is>
       </c>
       <c r="J21" s="1" t="n">
@@ -5575,7 +5575,7 @@
       </c>
       <c r="D22" s="1" t="inlineStr">
         <is>
-          <t>실무용 n8n 자동화 워크플로 9종 모음 — WhatsApp 에이전트, RAG 챗봇, 감성분석, 이메일 자동화, Airtable, 벡터 DB 파이프라인</t>
+          <t>A collection of 9 production n8n automation workflows - WhatsApp agent, RAG chatbot, sentiment analysis, email automation, Airtable, vector DB pipeline</t>
         </is>
       </c>
       <c r="E22" s="1" t="inlineStr">
@@ -5590,17 +5590,17 @@
       </c>
       <c r="G22" s="1" t="inlineStr">
         <is>
-          <t>1 에이전트 소프트웨어</t>
+          <t>1 Agent software</t>
         </is>
       </c>
       <c r="H22" s="1" t="inlineStr">
         <is>
-          <t>3 무관·판정불가</t>
+          <t>3 Unrelated/undecidable</t>
         </is>
       </c>
       <c r="I22" s="1" t="inlineStr">
         <is>
-          <t>2 학습·참고 자료</t>
+          <t>2 Learning/reference resource</t>
         </is>
       </c>
       <c r="J22" s="1" t="n">
@@ -5626,7 +5626,7 @@
       </c>
       <c r="D23" s="1" t="inlineStr">
         <is>
-          <t>KogniSwarm — GPT-4로 자율 AI 애플리케이션을 개발하는 Kotlin 오픈소스 프로젝트</t>
+          <t>KogniSwarm - an open-source Kotlin project for developing autonomous AI applications with GPT-4</t>
         </is>
       </c>
       <c r="E23" s="1" t="inlineStr">
@@ -5641,17 +5641,17 @@
       </c>
       <c r="G23" s="1" t="inlineStr">
         <is>
-          <t>3 무관·판정불가</t>
+          <t>3 Unrelated/undecidable</t>
         </is>
       </c>
       <c r="H23" s="1" t="inlineStr">
         <is>
-          <t>1 에이전트 소프트웨어</t>
+          <t>1 Agent software</t>
         </is>
       </c>
       <c r="I23" s="1" t="inlineStr">
         <is>
-          <t>1 에이전트 소프트웨어</t>
+          <t>1 Agent software</t>
         </is>
       </c>
       <c r="J23" s="1" t="n">
@@ -5677,7 +5677,7 @@
       </c>
       <c r="D24" s="1" t="inlineStr">
         <is>
-          <t>autogen을 이용한 실험 모음</t>
+          <t>A collection of experiments using autogen</t>
         </is>
       </c>
       <c r="E24" s="1" t="inlineStr">
@@ -5690,17 +5690,17 @@
       </c>
       <c r="G24" s="1" t="inlineStr">
         <is>
-          <t>1 에이전트 소프트웨어</t>
+          <t>1 Agent software</t>
         </is>
       </c>
       <c r="H24" s="1" t="inlineStr">
         <is>
-          <t>2 학습·참고 자료</t>
+          <t>2 Learning/reference resource</t>
         </is>
       </c>
       <c r="I24" s="1" t="inlineStr">
         <is>
-          <t>2 학습·참고 자료</t>
+          <t>2 Learning/reference resource</t>
         </is>
       </c>
       <c r="J24" s="1" t="n">
@@ -5726,7 +5726,7 @@
       </c>
       <c r="D25" s="1" t="inlineStr">
         <is>
-          <t>O2.services AI Hive(AI 에이전트 동적 군집)의 사업 문서·피치 자료</t>
+          <t>Business documents and pitch materials of O2.services AI Hive (a dynamic swarm of AI agents)</t>
         </is>
       </c>
       <c r="E25" s="1" t="inlineStr">
@@ -5739,17 +5739,17 @@
       </c>
       <c r="G25" s="1" t="inlineStr">
         <is>
-          <t>1 에이전트 소프트웨어</t>
+          <t>1 Agent software</t>
         </is>
       </c>
       <c r="H25" s="1" t="inlineStr">
         <is>
-          <t>2 학습·참고 자료</t>
+          <t>2 Learning/reference resource</t>
         </is>
       </c>
       <c r="I25" s="1" t="inlineStr">
         <is>
-          <t>2 학습·참고 자료</t>
+          <t>2 Learning/reference resource</t>
         </is>
       </c>
       <c r="J25" s="1" t="n">
@@ -5775,7 +5775,7 @@
       </c>
       <c r="D26" s="1" t="inlineStr">
         <is>
-          <t>개인화 AI 에이전트를 가장 빠르게 만드는 방법</t>
+          <t>The fastest way to build personalized AI agents</t>
         </is>
       </c>
       <c r="E26" s="1" t="inlineStr">
@@ -5790,17 +5790,17 @@
       </c>
       <c r="G26" s="1" t="inlineStr">
         <is>
-          <t>1 에이전트 소프트웨어</t>
+          <t>1 Agent software</t>
         </is>
       </c>
       <c r="H26" s="1" t="inlineStr">
         <is>
-          <t>3 무관·판정불가</t>
+          <t>3 Unrelated/undecidable</t>
         </is>
       </c>
       <c r="I26" s="1" t="inlineStr">
         <is>
-          <t>1 에이전트 소프트웨어</t>
+          <t>1 Agent software</t>
         </is>
       </c>
       <c r="J26" s="1" t="n">
@@ -5826,7 +5826,7 @@
       </c>
       <c r="D27" s="1" t="inlineStr">
         <is>
-          <t>SIGIR 2024 논문: TRAD — 단계별 사고 검색과 정렬된 의사결정으로 LLM 에이전트 강화</t>
+          <t>SIGIR 2024 paper: TRAD - enhancing LLM agents with step-wise thought retrieval and aligned decision making</t>
         </is>
       </c>
       <c r="E27" s="1" t="inlineStr">
@@ -5839,17 +5839,17 @@
       </c>
       <c r="G27" s="1" t="inlineStr">
         <is>
-          <t>1 에이전트 소프트웨어</t>
+          <t>1 Agent software</t>
         </is>
       </c>
       <c r="H27" s="1" t="inlineStr">
         <is>
-          <t>2 학습·참고 자료</t>
+          <t>2 Learning/reference resource</t>
         </is>
       </c>
       <c r="I27" s="1" t="inlineStr">
         <is>
-          <t>2 학습·참고 자료</t>
+          <t>2 Learning/reference resource</t>
         </is>
       </c>
       <c r="J27" s="1" t="n">
@@ -5875,7 +5875,7 @@
       </c>
       <c r="D28" s="1" t="inlineStr">
         <is>
-          <t>TianGong-Agent (설명 없음)</t>
+          <t>TianGong-Agent (no description)</t>
         </is>
       </c>
       <c r="E28" s="1" t="inlineStr">
@@ -5888,17 +5888,17 @@
       </c>
       <c r="G28" s="1" t="inlineStr">
         <is>
-          <t>1 에이전트 소프트웨어</t>
+          <t>1 Agent software</t>
         </is>
       </c>
       <c r="H28" s="1" t="inlineStr">
         <is>
-          <t>3 무관·판정불가</t>
+          <t>3 Unrelated/undecidable</t>
         </is>
       </c>
       <c r="I28" s="1" t="inlineStr">
         <is>
-          <t>1 에이전트 소프트웨어</t>
+          <t>1 Agent software</t>
         </is>
       </c>
       <c r="J28" s="1" t="n">
@@ -5924,7 +5924,7 @@
       </c>
       <c r="D29" s="1" t="inlineStr">
         <is>
-          <t>맞춤 에이전트 기능과 서브에이전트로 Claude Code를 만능 AI 에이전트로 만들기</t>
+          <t>Turning Claude Code into an all-purpose AI agent with custom agent features and sub-agents</t>
         </is>
       </c>
       <c r="E29" s="1" t="inlineStr">
@@ -5937,17 +5937,17 @@
       </c>
       <c r="G29" s="1" t="inlineStr">
         <is>
-          <t>1 에이전트 소프트웨어</t>
+          <t>1 Agent software</t>
         </is>
       </c>
       <c r="H29" s="1" t="inlineStr">
         <is>
-          <t>3 무관·판정불가</t>
+          <t>3 Unrelated/undecidable</t>
         </is>
       </c>
       <c r="I29" s="1" t="inlineStr">
         <is>
-          <t>1 에이전트 소프트웨어</t>
+          <t>1 Agent software</t>
         </is>
       </c>
       <c r="J29" s="1" t="n">
@@ -5973,7 +5973,7 @@
       </c>
       <c r="D30" s="1" t="inlineStr">
         <is>
-          <t>⚠️ 폐기됨(DEPRECATED) — coderag로 대체</t>
+          <t>⚠️ DEPRECATED - replaced by coderag</t>
         </is>
       </c>
       <c r="E30" s="1" t="inlineStr">
@@ -5988,17 +5988,17 @@
       </c>
       <c r="G30" s="1" t="inlineStr">
         <is>
-          <t>1 에이전트 소프트웨어</t>
+          <t>1 Agent software</t>
         </is>
       </c>
       <c r="H30" s="1" t="inlineStr">
         <is>
-          <t>3 무관·판정불가</t>
+          <t>3 Unrelated/undecidable</t>
         </is>
       </c>
       <c r="I30" s="1" t="inlineStr">
         <is>
-          <t>1 에이전트 소프트웨어</t>
+          <t>1 Agent software</t>
         </is>
       </c>
       <c r="J30" s="1" t="n">
@@ -6024,7 +6024,7 @@
       </c>
       <c r="D31" s="1" t="inlineStr">
         <is>
-          <t>MCP-Zero: 자율 LLM 에이전트를 위한 능동적 도구 탐색(논문)</t>
+          <t>MCP-Zero: active tool discovery for autonomous LLM agents (paper)</t>
         </is>
       </c>
       <c r="E31" s="1" t="inlineStr">
@@ -6037,17 +6037,17 @@
       </c>
       <c r="G31" s="1" t="inlineStr">
         <is>
-          <t>1 에이전트 소프트웨어</t>
+          <t>1 Agent software</t>
         </is>
       </c>
       <c r="H31" s="1" t="inlineStr">
         <is>
-          <t>2 학습·참고 자료</t>
+          <t>2 Learning/reference resource</t>
         </is>
       </c>
       <c r="I31" s="1" t="inlineStr">
         <is>
-          <t>2 학습·참고 자료</t>
+          <t>2 Learning/reference resource</t>
         </is>
       </c>
       <c r="J31" s="1" t="n">
@@ -6073,7 +6073,7 @@
       </c>
       <c r="D32" s="1" t="inlineStr">
         <is>
-          <t>Godot에서 Copilot을 쓰기 위한 마크다운 가이드라인(코딩 표준·워크플로 규칙)</t>
+          <t>Markdown guidelines for using Copilot in Godot (coding standards, workflow rules)</t>
         </is>
       </c>
       <c r="E32" s="1" t="inlineStr">
@@ -6088,17 +6088,17 @@
       </c>
       <c r="G32" s="1" t="inlineStr">
         <is>
-          <t>1 에이전트 소프트웨어</t>
+          <t>1 Agent software</t>
         </is>
       </c>
       <c r="H32" s="1" t="inlineStr">
         <is>
-          <t>2 학습·참고 자료</t>
+          <t>2 Learning/reference resource</t>
         </is>
       </c>
       <c r="I32" s="1" t="inlineStr">
         <is>
-          <t>1 에이전트 소프트웨어</t>
+          <t>1 Agent software</t>
         </is>
       </c>
       <c r="J32" s="1" t="n">
@@ -6124,7 +6124,7 @@
       </c>
       <c r="D33" s="1" t="inlineStr">
         <is>
-          <t>ToRA — 도구와 상호작용해 어려운 수학 추론 문제를 푸는 도구통합 LLM 에이전트 시리즈(ICLR'24 논문)</t>
+          <t>ToRA - a series of tool-integrated LLM agents that solve hard mathematical reasoning problems by interacting with tools (ICLR'24 paper)</t>
         </is>
       </c>
       <c r="E33" s="1" t="inlineStr">
@@ -6139,17 +6139,17 @@
       </c>
       <c r="G33" s="1" t="inlineStr">
         <is>
-          <t>1 에이전트 소프트웨어</t>
+          <t>1 Agent software</t>
         </is>
       </c>
       <c r="H33" s="1" t="inlineStr">
         <is>
-          <t>2 학습·참고 자료</t>
+          <t>2 Learning/reference resource</t>
         </is>
       </c>
       <c r="I33" s="1" t="inlineStr">
         <is>
-          <t>2 학습·참고 자료</t>
+          <t>2 Learning/reference resource</t>
         </is>
       </c>
       <c r="J33" s="1" t="n">
@@ -6175,7 +6175,7 @@
       </c>
       <c r="D34" s="1" t="inlineStr">
         <is>
-          <t>MCP를 배우며 만든 실용 가이드·클라이언트·서버 모음(학습용)</t>
+          <t>A collection of practical guides, clients, and servers made while learning MCP (for learning)</t>
         </is>
       </c>
       <c r="E34" s="1" t="inlineStr">
@@ -6190,17 +6190,17 @@
       </c>
       <c r="G34" s="1" t="inlineStr">
         <is>
-          <t>1 에이전트 소프트웨어</t>
+          <t>1 Agent software</t>
         </is>
       </c>
       <c r="H34" s="1" t="inlineStr">
         <is>
-          <t>2 학습·참고 자료</t>
+          <t>2 Learning/reference resource</t>
         </is>
       </c>
       <c r="I34" s="1" t="inlineStr">
         <is>
-          <t>2 학습·참고 자료</t>
+          <t>2 Learning/reference resource</t>
         </is>
       </c>
       <c r="J34" s="1" t="n">
@@ -6226,7 +6226,7 @@
       </c>
       <c r="D35" s="1" t="inlineStr">
         <is>
-          <t>대규모로 웹을 검색·스크랩·상호작용하는 컨텍스트 API</t>
+          <t>A context API for searching, scraping, and interacting with the web at scale</t>
         </is>
       </c>
       <c r="E35" s="1" t="inlineStr">
@@ -6241,17 +6241,17 @@
       </c>
       <c r="G35" s="1" t="inlineStr">
         <is>
-          <t>1 에이전트 소프트웨어</t>
+          <t>1 Agent software</t>
         </is>
       </c>
       <c r="H35" s="1" t="inlineStr">
         <is>
-          <t>3 무관·판정불가</t>
+          <t>3 Unrelated/undecidable</t>
         </is>
       </c>
       <c r="I35" s="1" t="inlineStr">
         <is>
-          <t>1 에이전트 소프트웨어</t>
+          <t>1 Agent software</t>
         </is>
       </c>
       <c r="J35" s="1" t="n">
@@ -6277,7 +6277,7 @@
       </c>
       <c r="D36" s="1" t="inlineStr">
         <is>
-          <t>Ecma TC-56 NLIP(자연어 상호작용 프로토콜) 관련 문서 저장소</t>
+          <t>A documentation repository for Ecma TC-56 NLIP (Natural Language Interaction Protocol)</t>
         </is>
       </c>
       <c r="E36" s="1" t="inlineStr">
@@ -6292,17 +6292,17 @@
       </c>
       <c r="G36" s="1" t="inlineStr">
         <is>
-          <t>1 에이전트 소프트웨어</t>
+          <t>1 Agent software</t>
         </is>
       </c>
       <c r="H36" s="1" t="inlineStr">
         <is>
-          <t>2 학습·참고 자료</t>
+          <t>2 Learning/reference resource</t>
         </is>
       </c>
       <c r="I36" s="1" t="inlineStr">
         <is>
-          <t>2 학습·참고 자료</t>
+          <t>2 Learning/reference resource</t>
         </is>
       </c>
       <c r="J36" s="1" t="n">
@@ -6328,7 +6328,7 @@
       </c>
       <c r="D37" s="1" t="inlineStr">
         <is>
-          <t>AI 에이전트 워크숍용 실습(랩) 저장소</t>
+          <t>A hands-on lab repository for an AI agent workshop</t>
         </is>
       </c>
       <c r="E37" s="1" t="inlineStr">
@@ -6341,17 +6341,17 @@
       </c>
       <c r="G37" s="1" t="inlineStr">
         <is>
-          <t>1 에이전트 소프트웨어</t>
+          <t>1 Agent software</t>
         </is>
       </c>
       <c r="H37" s="1" t="inlineStr">
         <is>
-          <t>2 학습·참고 자료</t>
+          <t>2 Learning/reference resource</t>
         </is>
       </c>
       <c r="I37" s="1" t="inlineStr">
         <is>
-          <t>2 학습·참고 자료</t>
+          <t>2 Learning/reference resource</t>
         </is>
       </c>
       <c r="J37" s="1" t="n">
@@ -6377,7 +6377,7 @@
       </c>
       <c r="D38" s="1" t="inlineStr">
         <is>
-          <t>MCP 서버 개발용 TypeScript 스타터 템플릿</t>
+          <t>A TypeScript starter template for developing MCP servers</t>
         </is>
       </c>
       <c r="E38" s="1" t="inlineStr">
@@ -6392,17 +6392,17 @@
       </c>
       <c r="G38" s="1" t="inlineStr">
         <is>
-          <t>1 에이전트 소프트웨어</t>
+          <t>1 Agent software</t>
         </is>
       </c>
       <c r="H38" s="1" t="inlineStr">
         <is>
-          <t>3 무관·판정불가</t>
+          <t>3 Unrelated/undecidable</t>
         </is>
       </c>
       <c r="I38" s="1" t="inlineStr">
         <is>
-          <t>1 에이전트 소프트웨어</t>
+          <t>1 Agent software</t>
         </is>
       </c>
       <c r="J38" s="1" t="n">
@@ -6428,7 +6428,7 @@
       </c>
       <c r="D39" s="1" t="inlineStr">
         <is>
-          <t>🐧 작업 중… (내용 없음)</t>
+          <t>🐧 Work in progress… (no content)</t>
         </is>
       </c>
       <c r="E39" s="1" t="inlineStr">
@@ -6443,17 +6443,17 @@
       </c>
       <c r="G39" s="1" t="inlineStr">
         <is>
-          <t>3 무관·판정불가</t>
+          <t>3 Unrelated/undecidable</t>
         </is>
       </c>
       <c r="H39" s="1" t="inlineStr">
         <is>
-          <t>3 무관·판정불가</t>
+          <t>3 Unrelated/undecidable</t>
         </is>
       </c>
       <c r="I39" s="1" t="inlineStr">
         <is>
-          <t>1 에이전트 소프트웨어</t>
+          <t>1 Agent software</t>
         </is>
       </c>
       <c r="J39" s="1" t="n">
@@ -6479,7 +6479,7 @@
       </c>
       <c r="D40" s="1" t="inlineStr">
         <is>
-          <t>Thordata 공식 개발자 포털 — 프록시 인프라·웹 데이터 도구·SDK·튜토리얼·AI 연동 개요</t>
+          <t>Thordata official developer portal - overview of proxy infrastructure, web data tools, SDKs, tutorials, and AI integrations</t>
         </is>
       </c>
       <c r="E40" s="1" t="inlineStr">
@@ -6494,17 +6494,17 @@
       </c>
       <c r="G40" s="1" t="inlineStr">
         <is>
-          <t>1 에이전트 소프트웨어</t>
+          <t>1 Agent software</t>
         </is>
       </c>
       <c r="H40" s="1" t="inlineStr">
         <is>
-          <t>2 학습·참고 자료</t>
+          <t>2 Learning/reference resource</t>
         </is>
       </c>
       <c r="I40" s="1" t="inlineStr">
         <is>
-          <t>2 학습·참고 자료</t>
+          <t>2 Learning/reference resource</t>
         </is>
       </c>
       <c r="J40" s="1" t="n">
@@ -6530,7 +6530,7 @@
       </c>
       <c r="D41" s="1" t="inlineStr">
         <is>
-          <t>Letta SDK(TypeScript·Python) 코드 스니펫 — 상태 유지 AI 에이전트 개발용</t>
+          <t>Code snippets for the Letta SDK (TypeScript, Python) - for developing stateful AI agents</t>
         </is>
       </c>
       <c r="E41" s="1" t="inlineStr">
@@ -6545,17 +6545,17 @@
       </c>
       <c r="G41" s="1" t="inlineStr">
         <is>
-          <t>1 에이전트 소프트웨어</t>
+          <t>1 Agent software</t>
         </is>
       </c>
       <c r="H41" s="1" t="inlineStr">
         <is>
-          <t>2 학습·참고 자료</t>
+          <t>2 Learning/reference resource</t>
         </is>
       </c>
       <c r="I41" s="1" t="inlineStr">
         <is>
-          <t>2 학습·참고 자료</t>
+          <t>2 Learning/reference resource</t>
         </is>
       </c>
       <c r="J41" s="1" t="n">

</xml_diff>